<commit_message>
Update welcome screen date layout and spin timing config
</commit_message>
<xml_diff>
--- a/danhsachkhachmoi.xlsx
+++ b/danhsachkhachmoi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\VinhPhuVinhPhuc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41A09B1-E7FC-4052-81F8-EF59BB365C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23131571-4863-4E9E-9022-87F383934C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
   <si>
     <t>STT</t>
   </si>
@@ -423,6 +423,12 @@
   </si>
   <si>
     <t>Đại lý Tâm Hương</t>
+  </si>
+  <si>
+    <t>Đại lý Hùng Phượng</t>
+  </si>
+  <si>
+    <t>Điện máy TC</t>
   </si>
 </sst>
 </file>
@@ -501,7 +507,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -522,6 +528,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1518,17 +1527,30 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65"/>
-      <c r="B65"/>
-      <c r="C65" s="7"/>
+      <c r="A65" s="5">
+        <v>64</v>
+      </c>
+      <c r="B65" s="5">
+        <v>64</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66"/>
-      <c r="B66"/>
+      <c r="A66" s="5">
+        <v>65</v>
+      </c>
+      <c r="B66" s="5">
+        <v>65</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67"/>
-      <c r="B67"/>
+      <c r="B67" s="5"/>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68"/>

</xml_diff>